<commit_message>
Referral log: settle Alfred Chan RM8,700 (Datuk Francis/D001 referral); decision note
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KYEhLFiAptb1SoFtQRsqbZ
</commit_message>
<xml_diff>
--- a/Referral_Fee_Log_Voucher_Receipt.xlsx
+++ b/Referral_Fee_Log_Voucher_Receipt.xlsx
@@ -619,7 +619,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5" ht="24" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
         <is>
@@ -627,7 +626,6 @@
         </is>
       </c>
     </row>
-    <row r="6"/>
     <row r="7" ht="30" customHeight="1">
       <c r="A7" s="4" t="inlineStr">
         <is>
@@ -783,13 +781,39 @@
         <f>IF(D10="","","PV/2026/"&amp;TEXT(A10,"000"))</f>
         <v/>
       </c>
-      <c r="C10" s="9" t="n"/>
-      <c r="D10" s="8" t="n"/>
-      <c r="E10" s="8" t="n"/>
-      <c r="F10" s="8" t="n"/>
-      <c r="G10" s="10" t="n"/>
-      <c r="H10" s="8" t="n"/>
-      <c r="I10" s="8" t="n"/>
+      <c r="C10" s="9" t="inlineStr">
+        <is>
+          <t>19/09/2026</t>
+        </is>
+      </c>
+      <c r="D10" s="8" t="inlineStr">
+        <is>
+          <t>Alfred Chan</t>
+        </is>
+      </c>
+      <c r="E10" s="8" t="inlineStr">
+        <is>
+          <t>xxxxxx-xx-xxxx</t>
+        </is>
+      </c>
+      <c r="F10" s="8" t="inlineStr">
+        <is>
+          <t>Datuk Francis — Hartamas Heights land (D001)</t>
+        </is>
+      </c>
+      <c r="G10" s="10" t="n">
+        <v>8700</v>
+      </c>
+      <c r="H10" s="8" t="inlineStr">
+        <is>
+          <t>M2U transfer</t>
+        </is>
+      </c>
+      <c r="I10" s="8" t="inlineStr">
+        <is>
+          <t>OR/2026/003</t>
+        </is>
+      </c>
       <c r="J10" s="10">
         <f>IF(G10="","",SUM($G$8:G10))</f>
         <v/>
@@ -1339,7 +1363,6 @@
       <c r="I36" s="8" t="n"/>
       <c r="J36" s="8" t="n"/>
     </row>
-    <row r="37"/>
     <row r="38">
       <c r="A38" s="13" t="inlineStr">
         <is>
@@ -1397,7 +1420,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5" ht="24" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
         <is>
@@ -1405,7 +1427,6 @@
         </is>
       </c>
     </row>
-    <row r="6"/>
     <row r="7">
       <c r="A7" s="14" t="inlineStr">
         <is>
@@ -1429,7 +1450,6 @@
         </is>
       </c>
     </row>
-    <row r="8"/>
     <row r="9">
       <c r="A9" s="14" t="inlineStr">
         <is>
@@ -1445,7 +1465,6 @@
       <c r="D9" s="22" t="n"/>
       <c r="E9" s="22" t="n"/>
     </row>
-    <row r="10"/>
     <row r="11">
       <c r="A11" s="14" t="inlineStr">
         <is>
@@ -1460,7 +1479,6 @@
       <c r="D11" s="22" t="n"/>
       <c r="E11" s="22" t="n"/>
     </row>
-    <row r="12"/>
     <row r="13">
       <c r="A13" s="14" t="n"/>
       <c r="B13" s="23" t="inlineStr"/>
@@ -1468,7 +1486,6 @@
       <c r="D13" s="22" t="n"/>
       <c r="E13" s="22" t="n"/>
     </row>
-    <row r="14"/>
     <row r="15">
       <c r="A15" s="16" t="inlineStr">
         <is>
@@ -1541,7 +1558,6 @@
       <c r="D19" s="17" t="n"/>
       <c r="E19" s="18" t="n"/>
     </row>
-    <row r="20"/>
     <row r="21">
       <c r="A21" s="14" t="inlineStr">
         <is>
@@ -1557,15 +1573,12 @@
       <c r="D21" s="22" t="n"/>
       <c r="E21" s="22" t="n"/>
     </row>
-    <row r="22"/>
     <row r="23">
       <c r="A23" s="14" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="14" t="n"/>
     </row>
-    <row r="25"/>
-    <row r="26"/>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
@@ -1600,7 +1613,6 @@
         </is>
       </c>
     </row>
-    <row r="29"/>
     <row r="30">
       <c r="A30" s="13" t="inlineStr">
         <is>
@@ -1668,7 +1680,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5" ht="24" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
         <is>
@@ -1676,7 +1687,6 @@
         </is>
       </c>
     </row>
-    <row r="6"/>
     <row r="7">
       <c r="A7" s="14" t="inlineStr">
         <is>
@@ -1700,7 +1710,6 @@
         </is>
       </c>
     </row>
-    <row r="8"/>
     <row r="9">
       <c r="A9" s="14" t="inlineStr">
         <is>
@@ -1716,7 +1725,6 @@
       <c r="D9" s="22" t="n"/>
       <c r="E9" s="22" t="n"/>
     </row>
-    <row r="10"/>
     <row r="11">
       <c r="A11" s="14" t="inlineStr">
         <is>
@@ -1735,7 +1743,6 @@
       <c r="D12" s="22" t="n"/>
       <c r="E12" s="22" t="n"/>
     </row>
-    <row r="13"/>
     <row r="14">
       <c r="A14" s="14" t="inlineStr">
         <is>
@@ -1747,7 +1754,6 @@
       </c>
       <c r="C14" s="18" t="n"/>
     </row>
-    <row r="15"/>
     <row r="16">
       <c r="A16" s="14" t="inlineStr">
         <is>
@@ -1763,13 +1769,9 @@
       <c r="D16" s="22" t="n"/>
       <c r="E16" s="22" t="n"/>
     </row>
-    <row r="17"/>
     <row r="18">
       <c r="A18" s="14" t="n"/>
     </row>
-    <row r="19"/>
-    <row r="20"/>
-    <row r="21"/>
     <row r="22">
       <c r="D22" t="inlineStr">
         <is>
@@ -1791,8 +1793,6 @@
         </is>
       </c>
     </row>
-    <row r="25"/>
-    <row r="26"/>
     <row r="27" ht="28" customHeight="1">
       <c r="A27" s="21" t="inlineStr">
         <is>

</xml_diff>